<commit_message>
Intro a Django, tutorial documentación oficial
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="65">
   <si>
     <t>Enlace</t>
   </si>
@@ -202,6 +202,18 @@
   </si>
   <si>
     <t>Tutorial y documentación w3</t>
+  </si>
+  <si>
+    <t>https://www.djangoproject.com/</t>
+  </si>
+  <si>
+    <t>Documentación oficial de Django</t>
+  </si>
+  <si>
+    <t>https://docs.djangoproject.com/en/6.0/intro/tutorial01/</t>
+  </si>
+  <si>
+    <t>Totorial introductoria a Django</t>
   </si>
 </sst>
 </file>
@@ -540,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C33"/>
+  <dimension ref="B2:C35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -798,6 +810,22 @@
       </c>
       <c r="C33" t="s">
         <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B34" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -833,8 +861,10 @@
     <hyperlink ref="B31" r:id="rId29"/>
     <hyperlink ref="B32" r:id="rId30"/>
     <hyperlink ref="B33" r:id="rId31"/>
+    <hyperlink ref="B34" r:id="rId32"/>
+    <hyperlink ref="B35" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId32"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId34"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ejemplos trabajo con plantillas
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
   <si>
     <t>Enlace</t>
   </si>
@@ -214,6 +214,12 @@
   </si>
   <si>
     <t>Totorial introductoria a Django</t>
+  </si>
+  <si>
+    <t>https://docs.djangoproject.com/en/6.0/topics/templates/#</t>
+  </si>
+  <si>
+    <t>Uso de plantillas en Django - Sintaxis</t>
   </si>
 </sst>
 </file>
@@ -552,7 +558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C35"/>
+  <dimension ref="B2:C36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -826,6 +832,14 @@
       </c>
       <c r="C35" t="s">
         <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -863,8 +877,9 @@
     <hyperlink ref="B33" r:id="rId31"/>
     <hyperlink ref="B34" r:id="rId32"/>
     <hyperlink ref="B35" r:id="rId33"/>
+    <hyperlink ref="B36" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId34"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId35"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Avance formulario de contacto
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="71">
   <si>
     <t>Enlace</t>
   </si>
@@ -220,6 +220,18 @@
   </si>
   <si>
     <t>Uso de plantillas en Django - Sintaxis</t>
+  </si>
+  <si>
+    <t>Formularios con Django</t>
+  </si>
+  <si>
+    <t>https://docs.djangoproject.com/en/6.0/topics/forms/</t>
+  </si>
+  <si>
+    <t>https://docs.djangoproject.com/en/6.0/ref/csrf/</t>
+  </si>
+  <si>
+    <t>csrf_token Django</t>
   </si>
 </sst>
 </file>
@@ -558,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C36"/>
+  <dimension ref="B2:C38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -840,6 +852,22 @@
       </c>
       <c r="C36" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B38" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C38" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -878,8 +906,10 @@
     <hyperlink ref="B34" r:id="rId32"/>
     <hyperlink ref="B35" r:id="rId33"/>
     <hyperlink ref="B36" r:id="rId34"/>
+    <hyperlink ref="B37" r:id="rId35"/>
+    <hyperlink ref="B38" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId35"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId37"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Incorporación de modelo compras
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="73">
   <si>
     <t>Enlace</t>
   </si>
@@ -232,6 +232,12 @@
   </si>
   <si>
     <t>csrf_token Django</t>
+  </si>
+  <si>
+    <t>https://docs.djangoproject.com/en/6.0/topics/db/models/</t>
+  </si>
+  <si>
+    <t>Modelos en Django</t>
   </si>
 </sst>
 </file>
@@ -570,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C38"/>
+  <dimension ref="B2:C39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -868,6 +874,14 @@
       </c>
       <c r="C38" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B39" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -908,8 +922,9 @@
     <hyperlink ref="B36" r:id="rId34"/>
     <hyperlink ref="B37" r:id="rId35"/>
     <hyperlink ref="B38" r:id="rId36"/>
+    <hyperlink ref="B39" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId37"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId38"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Edición y eleiminación de autores
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
   <si>
     <t>Enlace</t>
   </si>
@@ -244,6 +244,15 @@
   </si>
   <si>
     <t>Ejemplos de queries, filter</t>
+  </si>
+  <si>
+    <t>https://datatables.net/plug-ins/i18n/</t>
+  </si>
+  <si>
+    <t>Lenguajes Datatables, configuración</t>
+  </si>
+  <si>
+    <t>Librería similar a Datatables</t>
   </si>
 </sst>
 </file>
@@ -582,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C40"/>
+  <dimension ref="B2:C42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -896,6 +905,22 @@
       </c>
       <c r="C40" t="s">
         <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B41" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C41" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B42" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C42" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -938,8 +963,10 @@
     <hyperlink ref="B38" r:id="rId36"/>
     <hyperlink ref="B39" r:id="rId37"/>
     <hyperlink ref="B40" r:id="rId38"/>
+    <hyperlink ref="B41" r:id="rId39"/>
+    <hyperlink ref="B42" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId39"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId41"/>
 </worksheet>
 </file>
</xml_diff>